<commit_message>
feat: 0.6.0 categorias, check de enviado e log de erros no Drive
O histórico mostra um check nos itens confirmados pelo Sheets, conta as
notificações não vistas quando a lista está rolada e filtra por
categorias locais (NotificationCategorizer). No Code.gs, o destino fica
em SPREADSHEET_URL e SHEETS, e os erros vão para uma subpasta diária de
NotificaArquivo-Debug no Drive, sem token nem conteúdo das notificações.
</commit_message>
<xml_diff>
--- a/google-sheets/Modelo-Notifica-Arquivo.xlsx
+++ b/google-sheets/Modelo-Notifica-Arquivo.xlsx
@@ -2,11 +2,12 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Notificacoes" sheetId="1" r:id="Rd950cf19817543aa"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Categorias" sheetId="2" r:id="R7bca3bf8e08c4ea7"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Aplicativos" sheetId="3" r:id="Rbba4bd85e97044f8"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="4" r:id="R2bfa4f9430704a11"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Ajuda" sheetId="5" r:id="R29340c82af9f4cc9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Notificacoes" sheetId="1" r:id="R29d1264120bd4fb0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Categorias" sheetId="2" r:id="Rfc9cdbcbfb534d8b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Aplicativos" sheetId="3" r:id="R5e13507cd8ae4060"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="4" r:id="R2d85cc6d5c084591"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Ajuda" sheetId="5" r:id="R437a3c0c451f4b3d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Financeiro" sheetId="6" r:id="R7886eda56976474c"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -102,7 +103,7 @@
       <x:name val="Arial"/>
     </x:font>
   </x:fonts>
-  <x:fills count="7">
+  <x:fills count="9">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -134,8 +135,18 @@
         <x:fgColor rgb="FFFCE4E2"/>
       </x:patternFill>
     </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF157565"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFC6EFCE"/>
+      </x:patternFill>
+    </x:fill>
   </x:fills>
-  <x:borders count="7">
+  <x:borders count="9">
     <x:border/>
     <x:border>
       <x:left style="thin">
@@ -191,11 +202,21 @@
         <x:color rgb="FFD9E0DC"/>
       </x:bottom>
     </x:border>
+    <x:border>
+      <x:bottom style="thin">
+        <x:color rgb="FF63BE7B"/>
+      </x:bottom>
+    </x:border>
+    <x:border>
+      <x:top style="thin">
+        <x:color rgb="FF63BE7B"/>
+      </x:top>
+    </x:border>
   </x:borders>
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="84">
+  <x:cellXfs count="95">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <x:extLst>
@@ -388,6 +409,37 @@
     <x:xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment wrapText="1"/>
     </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="1" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="1" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="8" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="8" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1">
+      <x:extLst>
+        <x:ext uri="{C7286773-470A-42A8-94C5-96B5CB345126}">
+          <xfpb:xfComplement xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" i="0"/>
+        </x:ext>
+      </x:extLst>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="8" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="8" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1">
+      <x:extLst>
+        <x:ext uri="{C7286773-470A-42A8-94C5-96B5CB345126}">
+          <xfpb:xfComplement xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" i="0"/>
+        </x:ext>
+      </x:extLst>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="8" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="8" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1">
+      <x:extLst>
+        <x:ext uri="{C7286773-470A-42A8-94C5-96B5CB345126}">
+          <xfpb:xfComplement xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" i="0"/>
+        </x:ext>
+      </x:extLst>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="0" fillId="8" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="200" fontId="0" fillId="8" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
   </x:cellXfs>
   <x:cellStyles count="1">
     <x:cellStyle name="Normal" xfId="0"/>
@@ -399,7 +451,7 @@
         <x:color rgb="FF8B3A3A"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFCE4E2"/>
         </x:patternFill>
       </x:fill>
@@ -410,7 +462,7 @@
         <x:color rgb="FF9A5A20"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFFF0DF"/>
         </x:patternFill>
       </x:fill>
@@ -665,7 +717,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R1dba3acfa0364672"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R5644c530b34e43e6"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -695,7 +747,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R9bb3662e1aad46a9"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R16182a402d54497d"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -1299,7 +1351,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R53c2fcec45d74a7c"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc9dfba94ceb2411d"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -1433,7 +1485,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rbb58e198d0b042ec"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R96902cb9c8fb4a8d"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -1627,7 +1679,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7b5a999e9717424f"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc7e830aeeeaf473b"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2327,7 +2379,7 @@
     <x:mergeCell ref="A2:H2"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rebeef1561ef94344"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2723f84c07794c3c"/>
 </x:worksheet>
 </file>
 
@@ -2528,8 +2580,12 @@
       <x:c r="F15" s="62"/>
     </x:row>
     <x:row r="16">
-      <x:c r="A16" s="62"/>
-      <x:c r="B16" s="83"/>
+      <x:c r="A16" s="62" t="str">
+        <x:v>Financeiro</x:v>
+      </x:c>
+      <x:c r="B16" s="83" t="str">
+        <x:v>Copia automatica das notificacoes dos bancos escolhidos.</x:v>
+      </x:c>
       <x:c r="C16" s="62"/>
       <x:c r="D16" s="62"/>
       <x:c r="E16" s="62"/>
@@ -2566,4 +2622,199 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:sheetFormatPr defaultRowHeight="15"/>
+  <x:cols>
+    <x:col min="1" max="1" width="27.5" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="23.75" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="30" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="26.25" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="18.75" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="26.25" hidden="0" customWidth="1"/>
+    <x:col min="7" max="7" width="45" hidden="0" customWidth="1"/>
+    <x:col min="8" max="8" width="19.3799991607666" hidden="0" customWidth="1"/>
+    <x:col min="9" max="9" width="15" hidden="0" customWidth="1"/>
+    <x:col min="10" max="10" width="11.25" hidden="0" customWidth="1"/>
+    <x:col min="11" max="11" width="19.3799991607666" hidden="0" customWidth="1"/>
+  </x:cols>
+  <x:sheetData>
+    <x:row r="1" ht="24" customHeight="1">
+      <x:c r="A1" s="86" t="str">
+        <x:v>ID</x:v>
+      </x:c>
+      <x:c r="B1" s="86" t="str">
+        <x:v>Device ID</x:v>
+      </x:c>
+      <x:c r="C1" s="86" t="str">
+        <x:v>Chave fonte</x:v>
+      </x:c>
+      <x:c r="D1" s="86" t="str">
+        <x:v>Pacote</x:v>
+      </x:c>
+      <x:c r="E1" s="86" t="str">
+        <x:v>Aplicativo</x:v>
+      </x:c>
+      <x:c r="F1" s="86" t="str">
+        <x:v>Titulo</x:v>
+      </x:c>
+      <x:c r="G1" s="86" t="str">
+        <x:v>Texto</x:v>
+      </x:c>
+      <x:c r="H1" s="86" t="str">
+        <x:v>Data notificacao</x:v>
+      </x:c>
+      <x:c r="I1" s="86" t="str">
+        <x:v>Categoria</x:v>
+      </x:c>
+      <x:c r="J1" s="86" t="str">
+        <x:v>Sensivel?</x:v>
+      </x:c>
+      <x:c r="K1" s="86" t="str">
+        <x:v>Recebido em</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="2">
+      <x:c r="A2" s="89" t="str">
+        <x:v>EXEMPLO-003</x:v>
+      </x:c>
+      <x:c r="B2" s="89" t="str">
+        <x:v>xiaomi-redmi-note-6-pro</x:v>
+      </x:c>
+      <x:c r="C2" s="89" t="str">
+        <x:v>demo|nubank|1</x:v>
+      </x:c>
+      <x:c r="D2" s="89" t="str">
+        <x:v>com.nu.production</x:v>
+      </x:c>
+      <x:c r="E2" s="89" t="str">
+        <x:v>Nubank</x:v>
+      </x:c>
+      <x:c r="F2" s="89" t="str">
+        <x:v>Compra aprovada</x:v>
+      </x:c>
+      <x:c r="G2" s="89" t="str">
+        <x:v>Compra de exemplo - R$ 42,90</x:v>
+      </x:c>
+      <x:c r="H2" s="93" t="n">
+        <x:v>46250.958351608795</x:v>
+      </x:c>
+      <x:c r="I2" s="89" t="str">
+        <x:v>Financeiro</x:v>
+      </x:c>
+      <x:c r="J2" s="90" t="b">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="K2" s="93" t="n">
+        <x:v>46250.95904605324</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="3">
+      <x:c r="A3" s="91" t="str">
+        <x:v>EXEMPLO-004</x:v>
+      </x:c>
+      <x:c r="B3" s="91" t="str">
+        <x:v>xiaomi-redmi-note-6-pro</x:v>
+      </x:c>
+      <x:c r="C3" s="91" t="str">
+        <x:v>demo|nubank|2</x:v>
+      </x:c>
+      <x:c r="D3" s="91" t="str">
+        <x:v>com.nu.production</x:v>
+      </x:c>
+      <x:c r="E3" s="91" t="str">
+        <x:v>Nubank</x:v>
+      </x:c>
+      <x:c r="F3" s="91" t="str">
+        <x:v>Pix recebido</x:v>
+      </x:c>
+      <x:c r="G3" s="91" t="str">
+        <x:v>Transferencia demonstrativa</x:v>
+      </x:c>
+      <x:c r="H3" s="94" t="n">
+        <x:v>46250.923629386576</x:v>
+      </x:c>
+      <x:c r="I3" s="91" t="str">
+        <x:v>Financeiro</x:v>
+      </x:c>
+      <x:c r="J3" s="92" t="b">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="K3" s="94" t="n">
+        <x:v>46250.924323831015</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="4">
+      <x:c r="H4" s="6"/>
+      <x:c r="K4" s="6"/>
+    </x:row>
+    <x:row r="5">
+      <x:c r="H5" s="6"/>
+      <x:c r="K5" s="6"/>
+    </x:row>
+    <x:row r="6">
+      <x:c r="H6" s="6"/>
+      <x:c r="K6" s="6"/>
+    </x:row>
+    <x:row r="7">
+      <x:c r="H7" s="6"/>
+      <x:c r="K7" s="6"/>
+    </x:row>
+    <x:row r="8">
+      <x:c r="H8" s="6"/>
+      <x:c r="K8" s="6"/>
+    </x:row>
+    <x:row r="9">
+      <x:c r="H9" s="6"/>
+      <x:c r="K9" s="6"/>
+    </x:row>
+    <x:row r="10">
+      <x:c r="H10" s="6"/>
+      <x:c r="K10" s="6"/>
+    </x:row>
+    <x:row r="11">
+      <x:c r="H11" s="6"/>
+      <x:c r="K11" s="6"/>
+    </x:row>
+    <x:row r="12">
+      <x:c r="H12" s="6"/>
+      <x:c r="K12" s="6"/>
+    </x:row>
+    <x:row r="13">
+      <x:c r="H13" s="6"/>
+      <x:c r="K13" s="6"/>
+    </x:row>
+    <x:row r="14">
+      <x:c r="H14" s="6"/>
+      <x:c r="K14" s="6"/>
+    </x:row>
+    <x:row r="15">
+      <x:c r="H15" s="6"/>
+      <x:c r="K15" s="6"/>
+    </x:row>
+    <x:row r="16">
+      <x:c r="H16" s="6"/>
+      <x:c r="K16" s="6"/>
+    </x:row>
+    <x:row r="17">
+      <x:c r="H17" s="6"/>
+      <x:c r="K17" s="6"/>
+    </x:row>
+    <x:row r="18">
+      <x:c r="H18" s="6"/>
+      <x:c r="K18" s="6"/>
+    </x:row>
+    <x:row r="19">
+      <x:c r="H19" s="6"/>
+      <x:c r="K19" s="6"/>
+    </x:row>
+    <x:row r="20">
+      <x:c r="H20" s="6"/>
+      <x:c r="K20" s="6"/>
+    </x:row>
+  </x:sheetData>
+  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</x:worksheet>
 </file>
</xml_diff>